<commit_message>
Update AI Usage Report
</commit_message>
<xml_diff>
--- a/Template_PRJ301_AI_Usage_Report_Template.xlsx
+++ b/Template_PRJ301_AI_Usage_Report_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\PRJ---24-7-LLM-Tutor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PRJ301\PRJ---24-7-LLM-Tutor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A1E0F9-B63A-4F16-BBF8-F4C60A4E4054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4EE475-E647-4BB2-AD96-A73EA683F87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0.Overview" sheetId="1" r:id="rId1"/>
@@ -19,23 +19,12 @@
     <sheet name="2. Week n" sheetId="3" r:id="rId4"/>
     <sheet name="Instruction" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="129">
   <si>
     <t>PRJ301 - Project AI Usage Report</t>
   </si>
@@ -393,6 +382,42 @@
   </si>
   <si>
     <t>AI initially suggested overly complex UX flows, generated CSS with responsive overflow issues on smaller viewports, and lacked proper color contrast.</t>
+  </si>
+  <si>
+    <t>Design Use Case Diagram and 8 Use Case Specifications for the 24/7 LLM Tutor.</t>
+  </si>
+  <si>
+    <t>Generated the Use Case Diagram with 3 actors (Admin, Instructor, Student) and 8 use cases: UC01 Login &amp; Authorization, UC02 Manage User List, UC03 Manage Assignments, UC04 Submit ZIP &amp; SHA-256 Hashing, UC05 View Scores &amp; Feedback, UC06 Detect Error &amp; Initialize AI Session, UC07 Interact with 24/7 AI Tutor, and UC08 Get Personalized Learning Path. Generated detailed descriptions including main flows and exceptions for all 8 use cases.</t>
+  </si>
+  <si>
+    <t>Reviewed the generated use cases against the project requirements. Modified actor–use case relationships, use case names, main flows, and exception flows to match the AITA 24/7 LLM Tutor project.</t>
+  </si>
+  <si>
+    <t>3 actors, 8 use cases, 11 actor–use case associations, 8 detailed use case specifications</t>
+  </si>
+  <si>
+    <t>Some AI-generated use case relationships and descriptions may not fully match the project requirements and therefore required manual review and modification.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1_IiKnUxj3SQwrN2uhQHVUB0enmRgof_9?usp=sharing</t>
+  </si>
+  <si>
+    <t>Design Domain Model and ERD for the 24/7 LLM Tutor module</t>
+  </si>
+  <si>
+    <t>Generated a Domain Model and ERD structure for the core learning features, including Student, TutorConversation, TutorMessage, CodeError, LearningRecommendation, and LearningTopic, with suggested PK/FK relationships and cardinalities.</t>
+  </si>
+  <si>
+    <t>Compared the AI-generated model with the project Use Cases and requirements. Corrected entity responsibilities, PK/FK mapping, relationship cardinalities, and removed unnecessary attributes. Reviewed the model for 3NF consistency before preparing domain-model.md, erd.md, and README.md.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1Cv8UVkfH270j3_3KHpU-v4wu6AA63oxH?hl=vi</t>
+  </si>
+  <si>
+    <t>6 core entities; PK/FK and cardinalities defined; 3 documentation files prepared</t>
+  </si>
+  <si>
+    <t>AI initially suggested relationships and attributes that did not fully match the project's Use Cases. Manual review was required to correct cardinalities, foreign keys, and unnecessary data.</t>
   </si>
 </sst>
 </file>
@@ -549,7 +574,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -593,19 +618,40 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -919,99 +965,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.05" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="23">
         <v>4</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="27"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
@@ -1288,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1354,7 +1400,7 @@
       <c r="F2" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="11" t="s">
         <v>72</v>
       </c>
       <c r="H2" s="8" t="s">
@@ -1371,19 +1417,19 @@
       <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="15" t="s">
         <v>113</v>
       </c>
       <c r="G3" s="11" t="s">
@@ -1409,7 +1455,7 @@
       <c r="C4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="16" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="8" t="s">
@@ -1429,12 +1475,79 @@
       </c>
       <c r="J4" s="8" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="201.6">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="I5" s="8">
+        <v>4</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="144">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="8">
+        <v>5</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
     <hyperlink ref="G3" r:id="rId2" xr:uid="{88FF8E4D-AB20-4BD2-8574-82AFE88F9E13}"/>
+    <hyperlink ref="G2" r:id="rId3" xr:uid="{501F067C-697C-4220-A862-1205015787E2}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{54149B39-3898-44D3-B264-6816775C6CC8}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{0587752F-533C-4EAB-B92A-01C112087A94}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>